<commit_message>
docs: add Stage 2B current-law role map
</commit_message>
<xml_diff>
--- a/governance/risk_register.xlsx
+++ b/governance/risk_register.xlsx
@@ -214,27 +214,27 @@
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>medium</t>
+          <t>low</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>critical</t>
+          <t>major</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>P0</t>
+          <t>P1</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>DfT interaction classification and statutory route note required</t>
+          <t>Stage 2B role map distinguishes DfT engagement from Secretary of State confirmation; DfT procedural expectations still required</t>
         </is>
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>high</t>
+          <t>medium</t>
         </is>
       </c>
       <c r="I4" t="inlineStr">
@@ -244,7 +244,7 @@
       </c>
       <c r="J4" t="inlineStr">
         <is>
-          <t>2026-06-25</t>
+          <t>2026-06-26</t>
         </is>
       </c>
       <c r="K4" t="inlineStr">
@@ -254,7 +254,7 @@
       </c>
       <c r="L4" t="inlineStr">
         <is>
-          <t>open</t>
+          <t>controlled_open</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
docs: add Stage 2D Bristol decision route map
</commit_message>
<xml_diff>
--- a/governance/risk_register.xlsx
+++ b/governance/risk_register.xlsx
@@ -85,7 +85,7 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Bristol internal WPL order-making and statutory submission route unresolved after authority-status source chain narrowed</t>
+          <t>Bristol final WPL licensing-scheme order-maker and statutory submitter route unresolved</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
@@ -105,7 +105,7 @@
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>Stage 2C authority source-chain note narrows Bristol status but requires internal route map and Legal Review Agent sign-off</t>
+          <t>Stage 2D controls OBC progression and FBC member route but final order-making and Secretary of State submission require legal Monitoring Officer route confirmation</t>
         </is>
       </c>
       <c r="H2" t="inlineStr">
@@ -524,27 +524,27 @@
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>medium</t>
+          <t>low</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>critical</t>
+          <t>major</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>P0</t>
+          <t>P1</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>Decision notices and minutes acquired; assumptions register blocks implementation consultation FBC and preferred-scheme claims</t>
+          <t>Decision notices and minutes acquired; assumptions register and Stage 2D decision-route map block implementation consultation FBC order-making submission and preferred-scheme claims</t>
         </is>
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>medium</t>
+          <t>low</t>
         </is>
       </c>
       <c r="I9" t="inlineStr">
@@ -554,7 +554,7 @@
       </c>
       <c r="J9" t="inlineStr">
         <is>
-          <t>2026-06-25</t>
+          <t>2026-06-26</t>
         </is>
       </c>
       <c r="K9" t="inlineStr">
@@ -564,7 +564,7 @@
       </c>
       <c r="L9" t="inlineStr">
         <is>
-          <t>open</t>
+          <t>controlled_open</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
docs: add Stage 2E WECA role classification
</commit_message>
<xml_diff>
--- a/governance/risk_register.xlsx
+++ b/governance/risk_register.xlsx
@@ -147,7 +147,7 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>WECA MCA statutory role consent or assurance dependency misstated</t>
+          <t>WECA MCA statutory role consent funding assurance or no-role dependency misstated</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
@@ -167,7 +167,7 @@
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>Current law constitution and decision-record verification required</t>
+          <t>Stage 2E controls strategic-context and conditional funding-assurance wording but current-law role meeting-record search and funding dependency classification remain unresolved</t>
         </is>
       </c>
       <c r="H3" t="inlineStr">
@@ -182,7 +182,7 @@
       </c>
       <c r="J3" t="inlineStr">
         <is>
-          <t>2026-06-25</t>
+          <t>2026-06-26</t>
         </is>
       </c>
       <c r="K3" t="inlineStr">
@@ -192,7 +192,7 @@
       </c>
       <c r="L3" t="inlineStr">
         <is>
-          <t>open</t>
+          <t>narrowed_open</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
docs: add Stage 2H WECA funding assurance controls
</commit_message>
<xml_diff>
--- a/governance/risk_register.xlsx
+++ b/governance/risk_register.xlsx
@@ -167,7 +167,7 @@
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>Stage 2E controls strategic-context and conditional funding-assurance wording; Stage 2F controls that current scoped repo evidence does not identify WPL-specific transferred/concurrent WECA MCA order-making; Stage 2G bounded official ModernGov search did not locate formal WPL decision; no-role consent consultation-response and funding dependency conclusions remain unresolved</t>
+          <t>Stage 2E controls strategic-context and conditional funding-assurance wording; Stage 2F controls that current scoped repo evidence does not identify WPL-specific transferred/concurrent WECA MCA order-making; Stage 2G bounded official ModernGov search did not locate formal WPL decision; Stage 2H classifies package-level funding and assurance triggers; no-role consent consultation-response and final funding dependency conclusions remain unresolved</t>
         </is>
       </c>
       <c r="H3" t="inlineStr">
@@ -689,6 +689,68 @@
       <c r="L11" t="inlineStr">
         <is>
           <t>open</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>RISK-0011</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>Stage 2</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>Future agents overstate WECA MCA role because funding assurance context is scattered</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>major</t>
+        </is>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="G12" t="inlineStr">
+        <is>
+          <t>Post Stage 2H context packet bounded read rule and Stage 2H trigger map control future WECA MCA drafting</t>
+        </is>
+      </c>
+      <c r="H12" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="I12" t="inlineStr">
+        <is>
+          <t>Programme Orchestrator</t>
+        </is>
+      </c>
+      <c r="J12" t="inlineStr">
+        <is>
+          <t>2026-06-26</t>
+        </is>
+      </c>
+      <c r="K12" t="inlineStr">
+        <is>
+          <t>Simulation Gate Authority</t>
+        </is>
+      </c>
+      <c r="L12" t="inlineStr">
+        <is>
+          <t>controlled_open</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
docs: add Stage 2L context controls
</commit_message>
<xml_diff>
--- a/governance/risk_register.xlsx
+++ b/governance/risk_register.xlsx
@@ -725,12 +725,12 @@
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>Post Stage 2H context packet bounded read rule and Stage 2H trigger map control future WECA MCA drafting</t>
+          <t>Post Stage 2H context packet bounded read rule Stage 2H trigger map and Stage 2L context packet control future WECA MCA drafting</t>
         </is>
       </c>
       <c r="H12" t="inlineStr">
         <is>
-          <t>medium</t>
+          <t>low</t>
         </is>
       </c>
       <c r="I12" t="inlineStr">
@@ -749,6 +749,68 @@
         </is>
       </c>
       <c r="L12" t="inlineStr">
+        <is>
+          <t>controlled_open</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>RISK-0012</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>Stage 2</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>Future agents promote Stage 2 narrowing controls into OBC FBC consultation statutory submission or operations readiness because legal governance context is scattered</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>major</t>
+        </is>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="G13" t="inlineStr">
+        <is>
+          <t>Stage 2L mandatory context packet banned-claim list domain add-ons and subagent packet criteria control future legal governance statutory OBC FBC and consultation drafting</t>
+        </is>
+      </c>
+      <c r="H13" t="inlineStr">
+        <is>
+          <t>low</t>
+        </is>
+      </c>
+      <c r="I13" t="inlineStr">
+        <is>
+          <t>Programme Orchestrator</t>
+        </is>
+      </c>
+      <c r="J13" t="inlineStr">
+        <is>
+          <t>2026-06-26</t>
+        </is>
+      </c>
+      <c r="K13" t="inlineStr">
+        <is>
+          <t>Simulation Gate Authority</t>
+        </is>
+      </c>
+      <c r="L13" t="inlineStr">
         <is>
           <t>controlled_open</t>
         </is>

</xml_diff>

<commit_message>
docs: add Stage 4A spatial controls
</commit_message>
<xml_diff>
--- a/governance/risk_register.xlsx
+++ b/governance/risk_register.xlsx
@@ -291,7 +291,7 @@
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>Boundary manifest parking-base methodology and DPIA scope required</t>
+          <t>Stage 4A creates boundary manifest templates topology QA rules parking-base methodology canonical inventory headers DPIA scope and enforcement-linkage controls but no authoritative boundary or inventory data exists</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">
@@ -306,7 +306,7 @@
       </c>
       <c r="J5" t="inlineStr">
         <is>
-          <t>2026-06-25</t>
+          <t>2026-06-26</t>
         </is>
       </c>
       <c r="K5" t="inlineStr">
@@ -316,7 +316,7 @@
       </c>
       <c r="L5" t="inlineStr">
         <is>
-          <t>open</t>
+          <t>controlled_open</t>
         </is>
       </c>
     </row>
@@ -477,7 +477,7 @@
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>Licence and enforcement schemas added; operating procedures PCN templates and service policy still required</t>
+          <t>Licence and enforcement schemas added; Stage 4A inventory to enforcement linkage control added; operating procedures PCN templates and service policy still required</t>
         </is>
       </c>
       <c r="H8" t="inlineStr">
@@ -492,7 +492,7 @@
       </c>
       <c r="J8" t="inlineStr">
         <is>
-          <t>2026-06-25</t>
+          <t>2026-06-26</t>
         </is>
       </c>
       <c r="K8" t="inlineStr">

</xml_diff>

<commit_message>
docs: add Stage 5A appraisal controls
</commit_message>
<xml_diff>
--- a/governance/risk_register.xlsx
+++ b/governance/risk_register.xlsx
@@ -353,7 +353,7 @@
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>Stage-gate plan blocks OBC assembly</t>
+          <t>Stage 5A creates options OAR ASR ASST model-card uncertainty benefits transferability and reappraisal controls but no agreed ASR shortlist model output BCR VFM or OBC economic case exists</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
@@ -368,7 +368,7 @@
       </c>
       <c r="J6" t="inlineStr">
         <is>
-          <t>2026-06-25</t>
+          <t>2026-06-26</t>
         </is>
       </c>
       <c r="K6" t="inlineStr">
@@ -378,7 +378,7 @@
       </c>
       <c r="L6" t="inlineStr">
         <is>
-          <t>open</t>
+          <t>controlled_open</t>
         </is>
       </c>
     </row>
@@ -663,7 +663,7 @@
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>Source register labels landing pages and requires individual TAG units/source notes before modelling reliance</t>
+          <t>Source register labels landing pages and Stage 5A guidance-source requirements require individual TAG units databook source notes and VFM framework before method or VFM reliance</t>
         </is>
       </c>
       <c r="H11" t="inlineStr">
@@ -678,7 +678,7 @@
       </c>
       <c r="J11" t="inlineStr">
         <is>
-          <t>2026-06-25</t>
+          <t>2026-06-26</t>
         </is>
       </c>
       <c r="K11" t="inlineStr">
@@ -688,7 +688,7 @@
       </c>
       <c r="L11" t="inlineStr">
         <is>
-          <t>open</t>
+          <t>controlled_open</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
docs: add Stage 14C history rewrite dry run
</commit_message>
<xml_diff>
--- a/governance/risk_register.xlsx
+++ b/governance/risk_register.xlsx
@@ -1498,6 +1498,68 @@
         </is>
       </c>
     </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>RISK-0024</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>Stage 14C</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>Live history rewrite and force push disrupt existing clones branches pull requests or forks while still not guaranteeing hosted alert closure.</t>
+        </is>
+      </c>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="E25" t="inlineStr">
+        <is>
+          <t>major</t>
+        </is>
+      </c>
+      <c r="F25" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="G25" t="inlineStr">
+        <is>
+          <t>Stage 14C dry-run decision package helper script tested mirror rewrite refs/original deletion garbage collection redacted history scan and explicit-approval boundary.</t>
+        </is>
+      </c>
+      <c r="H25" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="I25" t="inlineStr">
+        <is>
+          <t>Public Release Review Agent</t>
+        </is>
+      </c>
+      <c r="J25" t="inlineStr">
+        <is>
+          <t>2026-06-26</t>
+        </is>
+      </c>
+      <c r="K25" t="inlineStr">
+        <is>
+          <t>Simulation Gate Authority</t>
+        </is>
+      </c>
+      <c r="L25" t="inlineStr">
+        <is>
+          <t>blocked_pending_explicit_approval</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
docs: record Stage 14D history rewrite completion
</commit_message>
<xml_diff>
--- a/governance/risk_register.xlsx
+++ b/governance/risk_register.xlsx
@@ -1531,12 +1531,12 @@
       </c>
       <c r="G25" t="inlineStr">
         <is>
-          <t>Stage 14C dry-run decision package helper script tested mirror rewrite refs/original deletion garbage collection redacted history scan and explicit-approval boundary.</t>
+          <t>Stage 14C dry-run controls were executed live in Stage 14D using force-with-lease, local all-history scan and fresh remote mirror scan; residual hosted alert forks caches and old clone risks remain tracked in RISK-0025.</t>
         </is>
       </c>
       <c r="H25" t="inlineStr">
         <is>
-          <t>medium</t>
+          <t>low</t>
         </is>
       </c>
       <c r="I25" t="inlineStr">
@@ -1556,7 +1556,69 @@
       </c>
       <c r="L25" t="inlineStr">
         <is>
-          <t>blocked_pending_explicit_approval</t>
+          <t>controlled_superseded_by_stage_14d</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>RISK-0025</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>Stage 14D</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>Post-rewrite users misinterpret repository-history remediation as GitGuardian closure, fork cleanup, cache purge or external token revocation.</t>
+        </is>
+      </c>
+      <c r="D26" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="E26" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="F26" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="G26" t="inlineStr">
+        <is>
+          <t>Stage 14D completion report records force-with-lease execution local all-history scan fresh remote mirror scan and explicit hosted-alert fork cache old-clone token caveats.</t>
+        </is>
+      </c>
+      <c r="H26" t="inlineStr">
+        <is>
+          <t>low</t>
+        </is>
+      </c>
+      <c r="I26" t="inlineStr">
+        <is>
+          <t>Public Release Review Agent</t>
+        </is>
+      </c>
+      <c r="J26" t="inlineStr">
+        <is>
+          <t>2026-06-26</t>
+        </is>
+      </c>
+      <c r="K26" t="inlineStr">
+        <is>
+          <t>Simulation Gate Authority</t>
+        </is>
+      </c>
+      <c r="L26" t="inlineStr">
+        <is>
+          <t>controlled_open</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
docs: add Stage 14E hosted alert disposition
</commit_message>
<xml_diff>
--- a/governance/risk_register.xlsx
+++ b/governance/risk_register.xlsx
@@ -1593,7 +1593,7 @@
       </c>
       <c r="G26" t="inlineStr">
         <is>
-          <t>Stage 14D completion report records force-with-lease execution local all-history scan fresh remote mirror scan and explicit hosted-alert fork cache old-clone token caveats.</t>
+          <t>Stage 14D completion report and Stage 14E hosted-alert disposition report record force-with-lease execution, local all-history scan, fresh remote mirror scan, GitHub secret-scanning disabled response, ggshield absence and explicit GitGuardian follow-up.</t>
         </is>
       </c>
       <c r="H26" t="inlineStr">
@@ -1618,7 +1618,69 @@
       </c>
       <c r="L26" t="inlineStr">
         <is>
-          <t>controlled_open</t>
+          <t>controlled_open_external_check_required</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>RISK-0026</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>Stage 14E</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>Future readers mistake repository-side verification for hosted GitGuardian closure.</t>
+        </is>
+      </c>
+      <c r="D27" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="E27" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="F27" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="G27" t="inlineStr">
+        <is>
+          <t>Stage 14E report records ggshield absence GitHub secret scanning disabled API response repo scans and explicit GitGuardian follow-up requirement.</t>
+        </is>
+      </c>
+      <c r="H27" t="inlineStr">
+        <is>
+          <t>low</t>
+        </is>
+      </c>
+      <c r="I27" t="inlineStr">
+        <is>
+          <t>Public Release Review Agent</t>
+        </is>
+      </c>
+      <c r="J27" t="inlineStr">
+        <is>
+          <t>2026-06-26</t>
+        </is>
+      </c>
+      <c r="K27" t="inlineStr">
+        <is>
+          <t>Simulation Gate Authority</t>
+        </is>
+      </c>
+      <c r="L27" t="inlineStr">
+        <is>
+          <t>controlled_open_external_check_required</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
docs: add Stage 15A source note expansion
</commit_message>
<xml_diff>
--- a/governance/risk_register.xlsx
+++ b/governance/risk_register.xlsx
@@ -1684,6 +1684,68 @@
         </is>
       </c>
     </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>RISK-0027</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>Stage 15A</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>Expanded source-note coverage is mistaken for complete evidence review or legal/gate sign-off</t>
+        </is>
+      </c>
+      <c r="D28" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="E28" t="inlineStr">
+        <is>
+          <t>major</t>
+        </is>
+      </c>
+      <c r="F28" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="G28" t="inlineStr">
+        <is>
+          <t>Stage 15A expanded notes, coverage register, extraction-manifest checks, raw-omitted wording checks, source-note QA, no-go wording, peer review and stage gate report preserve cohort boundary and keep ISS-0007 EG-0024 and EG-0038 open.</t>
+        </is>
+      </c>
+      <c r="H28" t="inlineStr">
+        <is>
+          <t>low</t>
+        </is>
+      </c>
+      <c r="I28" t="inlineStr">
+        <is>
+          <t>Evidence Librarian</t>
+        </is>
+      </c>
+      <c r="J28" t="inlineStr">
+        <is>
+          <t>2026-06-26</t>
+        </is>
+      </c>
+      <c r="K28" t="inlineStr">
+        <is>
+          <t>Simulation Gate Authority</t>
+        </is>
+      </c>
+      <c r="L28" t="inlineStr">
+        <is>
+          <t>controlled_open</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
docs: complete Stage 15B source notes
</commit_message>
<xml_diff>
--- a/governance/risk_register.xlsx
+++ b/governance/risk_register.xlsx
@@ -1746,6 +1746,68 @@
         </is>
       </c>
     </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>RISK-0028</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>Stage 15B</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>Acquired-priority source-note coverage completion wording leaks into OBC FBC statutory consultation legal or appraisal readiness claims</t>
+        </is>
+      </c>
+      <c r="D29" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="E29" t="inlineStr">
+        <is>
+          <t>major</t>
+        </is>
+      </c>
+      <c r="F29" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="G29" t="inlineStr">
+        <is>
+          <t>Stage 15B notes, coverage register, validator, gate report and public/officer wording qualify completion as acquired-priority source-note coverage only; EG-0044 preserves claim-level summary gap.</t>
+        </is>
+      </c>
+      <c r="H29" t="inlineStr">
+        <is>
+          <t>low</t>
+        </is>
+      </c>
+      <c r="I29" t="inlineStr">
+        <is>
+          <t>Evidence Librarian</t>
+        </is>
+      </c>
+      <c r="J29" t="inlineStr">
+        <is>
+          <t>2026-06-26</t>
+        </is>
+      </c>
+      <c r="K29" t="inlineStr">
+        <is>
+          <t>Simulation Gate Authority</t>
+        </is>
+      </c>
+      <c r="L29" t="inlineStr">
+        <is>
+          <t>controlled_open</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
docs: add Stage 16A claim summaries
</commit_message>
<xml_diff>
--- a/governance/risk_register.xlsx
+++ b/governance/risk_register.xlsx
@@ -1808,6 +1808,68 @@
         </is>
       </c>
     </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>RISK-0029</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>Stage 16A</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>Claim-summary completion wording leaks into claim truth OBC/FBC readiness legal clearance or statutory readiness</t>
+        </is>
+      </c>
+      <c r="D30" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="E30" t="inlineStr">
+        <is>
+          <t>major</t>
+        </is>
+      </c>
+      <c r="F30" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="G30" t="inlineStr">
+        <is>
+          <t>Stage 16A claim-summary register no-go register validator per-claim Markdown summaries public/officer wording and gate report preserve current-matrix-only status and EG-0045 future-claim gap.</t>
+        </is>
+      </c>
+      <c r="H30" t="inlineStr">
+        <is>
+          <t>low</t>
+        </is>
+      </c>
+      <c r="I30" t="inlineStr">
+        <is>
+          <t>Evidence/Citation Agent</t>
+        </is>
+      </c>
+      <c r="J30" t="inlineStr">
+        <is>
+          <t>2026-06-26</t>
+        </is>
+      </c>
+      <c r="K30" t="inlineStr">
+        <is>
+          <t>Simulation Gate Authority</t>
+        </is>
+      </c>
+      <c r="L30" t="inlineStr">
+        <is>
+          <t>controlled_open</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
docs: add Stage 17A authoring guardrails
</commit_message>
<xml_diff>
--- a/governance/risk_register.xlsx
+++ b/governance/risk_register.xlsx
@@ -1870,6 +1870,68 @@
         </is>
       </c>
     </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>RISK-0030</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>Stage 17A</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>Editable output wording leaks into assembled OBC FBC statutory consultation officer-review or authored PDF readiness claims</t>
+        </is>
+      </c>
+      <c r="D31" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="E31" t="inlineStr">
+        <is>
+          <t>major</t>
+        </is>
+      </c>
+      <c r="F31" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="G31" t="inlineStr">
+        <is>
+          <t>Stage 17A output register authoring README visual map fail-closed assembly scripts no-PDF checks statutory blocked-row checks public/officer wording and authoring QA preserve control-only status.</t>
+        </is>
+      </c>
+      <c r="H31" t="inlineStr">
+        <is>
+          <t>low</t>
+        </is>
+      </c>
+      <c r="I31" t="inlineStr">
+        <is>
+          <t>Technical Editor Agent</t>
+        </is>
+      </c>
+      <c r="J31" t="inlineStr">
+        <is>
+          <t>2026-06-26</t>
+        </is>
+      </c>
+      <c r="K31" t="inlineStr">
+        <is>
+          <t>Simulation Gate Authority</t>
+        </is>
+      </c>
+      <c r="L31" t="inlineStr">
+        <is>
+          <t>controlled_open</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
docs: add Stage 18A Nottingham transferability controls
</commit_message>
<xml_diff>
--- a/governance/risk_register.xlsx
+++ b/governance/risk_register.xlsx
@@ -1932,6 +1932,68 @@
         </is>
       </c>
     </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>RISK-0031</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>Stage 18A</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>Comparator lessons are treated as transferable Bristol evidence or ready parking mitigation</t>
+        </is>
+      </c>
+      <c r="D32" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="E32" t="inlineStr">
+        <is>
+          <t>major</t>
+        </is>
+      </c>
+      <c r="F32" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="G32" t="inlineStr">
+        <is>
+          <t>Stage 18A adds blocked NLR-0007 to NLR-0015 controls displacement checklist transferability-matrix hardening officer/public wording and validator cross-register checks</t>
+        </is>
+      </c>
+      <c r="H32" t="inlineStr">
+        <is>
+          <t>low</t>
+        </is>
+      </c>
+      <c r="I32" t="inlineStr">
+        <is>
+          <t>Comparator Evidence Agent</t>
+        </is>
+      </c>
+      <c r="J32" t="inlineStr">
+        <is>
+          <t>2026-06-26</t>
+        </is>
+      </c>
+      <c r="K32" t="inlineStr">
+        <is>
+          <t>Simulation Gate Authority</t>
+        </is>
+      </c>
+      <c r="L32" t="inlineStr">
+        <is>
+          <t>controlled_open</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
docs: add Stage 19A public comprehension controls
</commit_message>
<xml_diff>
--- a/governance/risk_register.xlsx
+++ b/governance/risk_register.xlsx
@@ -1994,6 +1994,68 @@
         </is>
       </c>
     </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>RISK-0032</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>Stage 19A</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>Public or cabinet navigation material is mistaken for professional assurance official council approval or WPL readiness</t>
+        </is>
+      </c>
+      <c r="D33" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="E33" t="inlineStr">
+        <is>
+          <t>major</t>
+        </is>
+      </c>
+      <c r="F33" t="inlineStr">
+        <is>
+          <t>P1</t>
+        </is>
+      </c>
+      <c r="G33" t="inlineStr">
+        <is>
+          <t>Stage 19A adds public and cabinet guides risk-control crosswalk visual RAG legend stage taxonomy and comprehension validator</t>
+        </is>
+      </c>
+      <c r="H33" t="inlineStr">
+        <is>
+          <t>low</t>
+        </is>
+      </c>
+      <c r="I33" t="inlineStr">
+        <is>
+          <t>Public Officer Review Agent</t>
+        </is>
+      </c>
+      <c r="J33" t="inlineStr">
+        <is>
+          <t>2026-06-26</t>
+        </is>
+      </c>
+      <c r="K33" t="inlineStr">
+        <is>
+          <t>Simulation Gate Authority</t>
+        </is>
+      </c>
+      <c r="L33" t="inlineStr">
+        <is>
+          <t>controlled_open</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
docs: add Stage 20A visual accessibility controls
</commit_message>
<xml_diff>
--- a/governance/risk_register.xlsx
+++ b/governance/risk_register.xlsx
@@ -2056,6 +2056,68 @@
         </is>
       </c>
     </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>RISK-0033</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>Stage 20A</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>Static visual source checks are mistaken for rendered accessibility review user testing WCAG certification or reader comprehension evidence</t>
+        </is>
+      </c>
+      <c r="D34" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="E34" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="F34" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="G34" t="inlineStr">
+        <is>
+          <t>Stage 20A adds visual QA register Mermaid captions legends text fallback references and validator output that states repo-level control only</t>
+        </is>
+      </c>
+      <c r="H34" t="inlineStr">
+        <is>
+          <t>low</t>
+        </is>
+      </c>
+      <c r="I34" t="inlineStr">
+        <is>
+          <t>Visual Map Review Agent</t>
+        </is>
+      </c>
+      <c r="J34" t="inlineStr">
+        <is>
+          <t>2026-06-26</t>
+        </is>
+      </c>
+      <c r="K34" t="inlineStr">
+        <is>
+          <t>Simulation Gate Authority</t>
+        </is>
+      </c>
+      <c r="L34" t="inlineStr">
+        <is>
+          <t>controlled_open</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
docs: add Stage 21A navigation integrity controls
</commit_message>
<xml_diff>
--- a/governance/risk_register.xlsx
+++ b/governance/risk_register.xlsx
@@ -2118,6 +2118,68 @@
         </is>
       </c>
     </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>RISK-0034</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>Stage 21A</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>Navigation integrity checks are mistaken for external URL liveness content correctness evidence accuracy accessibility assurance or WPL readiness</t>
+        </is>
+      </c>
+      <c r="D35" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="E35" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="F35" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="G35" t="inlineStr">
+        <is>
+          <t>Stage 21A adds repo-local link resolution latest-stage alignment required-route checks and explicit validator output limiting scope</t>
+        </is>
+      </c>
+      <c r="H35" t="inlineStr">
+        <is>
+          <t>low</t>
+        </is>
+      </c>
+      <c r="I35" t="inlineStr">
+        <is>
+          <t>Navigation Integrity Agent</t>
+        </is>
+      </c>
+      <c r="J35" t="inlineStr">
+        <is>
+          <t>2026-06-26</t>
+        </is>
+      </c>
+      <c r="K35" t="inlineStr">
+        <is>
+          <t>Simulation Gate Authority</t>
+        </is>
+      </c>
+      <c r="L35" t="inlineStr">
+        <is>
+          <t>controlled_open</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
docs: add Stage 22A source liveness controls
</commit_message>
<xml_diff>
--- a/governance/risk_register.xlsx
+++ b/governance/risk_register.xlsx
@@ -2180,6 +2180,68 @@
         </is>
       </c>
     </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>RISK-0035</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>Stage 22A</t>
+        </is>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>URL reachability and freshness metadata are mistaken for evidence truth source authority legal currentness source adequacy or WPL readiness</t>
+        </is>
+      </c>
+      <c r="D36" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="E36" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="F36" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="G36" t="inlineStr">
+        <is>
+          <t>Stage 22A uses reachable wording explicit metadata-only validator output public source-link page redirect visibility and register trail preserving EG-0049 and EG-0050</t>
+        </is>
+      </c>
+      <c r="H36" t="inlineStr">
+        <is>
+          <t>low</t>
+        </is>
+      </c>
+      <c r="I36" t="inlineStr">
+        <is>
+          <t>Source Liveness Agent</t>
+        </is>
+      </c>
+      <c r="J36" t="inlineStr">
+        <is>
+          <t>2026-06-26</t>
+        </is>
+      </c>
+      <c r="K36" t="inlineStr">
+        <is>
+          <t>Simulation Gate Authority</t>
+        </is>
+      </c>
+      <c r="L36" t="inlineStr">
+        <is>
+          <t>controlled_open</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
docs: add Stage 23A register reference controls
</commit_message>
<xml_diff>
--- a/governance/risk_register.xlsx
+++ b/governance/risk_register.xlsx
@@ -2242,6 +2242,68 @@
         </is>
       </c>
     </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>RISK-0036</t>
+        </is>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>Stage 23A</t>
+        </is>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>Resolved register IDs and paths are mistaken for row correctness evidence support mitigation adequacy professional assurance or WPL readiness</t>
+        </is>
+      </c>
+      <c r="D37" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="E37" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="F37" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="G37" t="inlineStr">
+        <is>
+          <t>Stage 23A uses scoped reference checks primary-key uniqueness checks linkage-only gate wording and EG-0051 residual gap</t>
+        </is>
+      </c>
+      <c r="H37" t="inlineStr">
+        <is>
+          <t>low</t>
+        </is>
+      </c>
+      <c r="I37" t="inlineStr">
+        <is>
+          <t>Register Reference Agent</t>
+        </is>
+      </c>
+      <c r="J37" t="inlineStr">
+        <is>
+          <t>2026-06-26</t>
+        </is>
+      </c>
+      <c r="K37" t="inlineStr">
+        <is>
+          <t>Simulation Gate Authority</t>
+        </is>
+      </c>
+      <c r="L37" t="inlineStr">
+        <is>
+          <t>controlled_open</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
docs: add Stage 24A dashboard consistency controls
</commit_message>
<xml_diff>
--- a/governance/risk_register.xlsx
+++ b/governance/risk_register.xlsx
@@ -2304,6 +2304,68 @@
         </is>
       </c>
     </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>RISK-0037</t>
+        </is>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>Stage 24A</t>
+        </is>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>Visible dashboard blocker consistency is mistaken for exhaustive blocker coverage risk adequacy mitigation adequacy or WPL readiness</t>
+        </is>
+      </c>
+      <c r="D38" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="E38" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="F38" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="G38" t="inlineStr">
+        <is>
+          <t>Stage 24A validates README blocker IDs current-stage surfacing dashboard wording and map references with blocker-surfacing-only caveats</t>
+        </is>
+      </c>
+      <c r="H38" t="inlineStr">
+        <is>
+          <t>low</t>
+        </is>
+      </c>
+      <c r="I38" t="inlineStr">
+        <is>
+          <t>Dashboard Consistency Agent</t>
+        </is>
+      </c>
+      <c r="J38" t="inlineStr">
+        <is>
+          <t>2026-06-26</t>
+        </is>
+      </c>
+      <c r="K38" t="inlineStr">
+        <is>
+          <t>Simulation Gate Authority</t>
+        </is>
+      </c>
+      <c r="L38" t="inlineStr">
+        <is>
+          <t>controlled_open</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
docs: add Stage 25A gate report structure controls
</commit_message>
<xml_diff>
--- a/governance/risk_register.xlsx
+++ b/governance/risk_register.xlsx
@@ -2366,6 +2366,68 @@
         </is>
       </c>
     </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>RISK-0038</t>
+        </is>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>Stage 25A</t>
+        </is>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>Report structure checks are mistaken for historical command execution substantive gate correctness evidence truth or WPL readiness</t>
+        </is>
+      </c>
+      <c r="D39" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="E39" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="F39" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="G39" t="inlineStr">
+        <is>
+          <t>Stage 25A validates recent reports for focused commands full validation commands blocker sections gate decision sections and no-overclaim language with structure-only caveats</t>
+        </is>
+      </c>
+      <c r="H39" t="inlineStr">
+        <is>
+          <t>low</t>
+        </is>
+      </c>
+      <c r="I39" t="inlineStr">
+        <is>
+          <t>Gate Report Consistency Agent</t>
+        </is>
+      </c>
+      <c r="J39" t="inlineStr">
+        <is>
+          <t>2026-06-26</t>
+        </is>
+      </c>
+      <c r="K39" t="inlineStr">
+        <is>
+          <t>Simulation Gate Authority</t>
+        </is>
+      </c>
+      <c r="L39" t="inlineStr">
+        <is>
+          <t>controlled_open</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
docs: add Stage 26A validation evidence log controls
</commit_message>
<xml_diff>
--- a/governance/risk_register.xlsx
+++ b/governance/risk_register.xlsx
@@ -2428,6 +2428,68 @@
         </is>
       </c>
     </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>RISK-0039</t>
+        </is>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>Stage 26A</t>
+        </is>
+      </c>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>Validation logs are mistaken for evidence truth source currentness professional assurance substantive gate correctness or WPL readiness</t>
+        </is>
+      </c>
+      <c r="D40" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="E40" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="F40" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="G40" t="inlineStr">
+        <is>
+          <t>Stage 26A records command text run date commit reference exit code output summary evidence file and scope limits with explicit log-only caveats</t>
+        </is>
+      </c>
+      <c r="H40" t="inlineStr">
+        <is>
+          <t>low</t>
+        </is>
+      </c>
+      <c r="I40" t="inlineStr">
+        <is>
+          <t>Validation Evidence Agent</t>
+        </is>
+      </c>
+      <c r="J40" t="inlineStr">
+        <is>
+          <t>2026-06-26</t>
+        </is>
+      </c>
+      <c r="K40" t="inlineStr">
+        <is>
+          <t>Simulation Gate Authority</t>
+        </is>
+      </c>
+      <c r="L40" t="inlineStr">
+        <is>
+          <t>controlled_open</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
docs: add Stage 27A validation coverage controls
</commit_message>
<xml_diff>
--- a/governance/risk_register.xlsx
+++ b/governance/risk_register.xlsx
@@ -2490,6 +2490,68 @@
         </is>
       </c>
     </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>RISK-0040</t>
+        </is>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>Stage 27A</t>
+        </is>
+      </c>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>Validation coverage checks are mistaken for command authenticity command sufficiency evidence truth professional assurance or WPL readiness</t>
+        </is>
+      </c>
+      <c r="D41" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="E41" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="F41" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="G41" t="inlineStr">
+        <is>
+          <t>Stage 27A targets Stage 26A as lag-one coverage only and requires no-overclaim wording in rows logs and gate report</t>
+        </is>
+      </c>
+      <c r="H41" t="inlineStr">
+        <is>
+          <t>low</t>
+        </is>
+      </c>
+      <c r="I41" t="inlineStr">
+        <is>
+          <t>Validation Coverage Agent</t>
+        </is>
+      </c>
+      <c r="J41" t="inlineStr">
+        <is>
+          <t>2026-06-26</t>
+        </is>
+      </c>
+      <c r="K41" t="inlineStr">
+        <is>
+          <t>Simulation Gate Authority</t>
+        </is>
+      </c>
+      <c r="L41" t="inlineStr">
+        <is>
+          <t>controlled_open</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
docs: add Stage 28A Bristol public source controls
</commit_message>
<xml_diff>
--- a/governance/risk_register.xlsx
+++ b/governance/risk_register.xlsx
@@ -2552,6 +2552,68 @@
         </is>
       </c>
     </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>RISK-0041</t>
+        </is>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>Stage 28A</t>
+        </is>
+      </c>
+      <c r="C42" t="inlineStr">
+        <is>
+          <t>Bristol public-source coverage is mistaken for source authority currentness formal approval press or media accuracy or decision-grade sufficiency</t>
+        </is>
+      </c>
+      <c r="D42" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="E42" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="F42" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="G42" t="inlineStr">
+        <is>
+          <t>Stage 28A records source type access state repository status source-note status claim-use limits and no-formal-decision controls for the selected Bristol public-source cohort</t>
+        </is>
+      </c>
+      <c r="H42" t="inlineStr">
+        <is>
+          <t>low</t>
+        </is>
+      </c>
+      <c r="I42" t="inlineStr">
+        <is>
+          <t>Bristol Public Source Agent</t>
+        </is>
+      </c>
+      <c r="J42" t="inlineStr">
+        <is>
+          <t>2026-06-27</t>
+        </is>
+      </c>
+      <c r="K42" t="inlineStr">
+        <is>
+          <t>Simulation Gate Authority</t>
+        </is>
+      </c>
+      <c r="L42" t="inlineStr">
+        <is>
+          <t>controlled_open</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
docs: add Stage 29A subagent context controls
</commit_message>
<xml_diff>
--- a/governance/risk_register.xlsx
+++ b/governance/risk_register.xlsx
@@ -2614,6 +2614,68 @@
         </is>
       </c>
     </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t>RISK-0042</t>
+        </is>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>Stage 29A</t>
+        </is>
+      </c>
+      <c r="C43" t="inlineStr">
+        <is>
+          <t>Bounded subagent packets and validators are mistaken for proof that agents had complete context avoided hallucination or gave assurance-grade findings</t>
+        </is>
+      </c>
+      <c r="D43" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="E43" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="F43" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="G43" t="inlineStr">
+        <is>
+          <t>Require packet manifests banned claims explicit file limits synthesis disposition sign-off limitations and validator output caveats</t>
+        </is>
+      </c>
+      <c r="H43" t="inlineStr">
+        <is>
+          <t>low</t>
+        </is>
+      </c>
+      <c r="I43" t="inlineStr">
+        <is>
+          <t>Context Control Agent</t>
+        </is>
+      </c>
+      <c r="J43" t="inlineStr">
+        <is>
+          <t>2026-06-27</t>
+        </is>
+      </c>
+      <c r="K43" t="inlineStr">
+        <is>
+          <t>Simulation Gate Authority</t>
+        </is>
+      </c>
+      <c r="L43" t="inlineStr">
+        <is>
+          <t>controlled_open</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
docs: add Stage 30A validation coverage controls
</commit_message>
<xml_diff>
--- a/governance/risk_register.xlsx
+++ b/governance/risk_register.xlsx
@@ -2676,6 +2676,68 @@
         </is>
       </c>
     </row>
+    <row r="44">
+      <c r="A44" t="inlineStr">
+        <is>
+          <t>RISK-0043</t>
+        </is>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>Stage 30A</t>
+        </is>
+      </c>
+      <c r="C44" t="inlineStr">
+        <is>
+          <t>Validation coverage for Stage 29A is mistaken for command sufficiency command authenticity future agent compliance or readiness evidence</t>
+        </is>
+      </c>
+      <c r="D44" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="E44" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="F44" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="G44" t="inlineStr">
+        <is>
+          <t>Require lagged coverage wording Stage 29A repository-state caveat issue and gap links no-overclaim terms and gate report limitations</t>
+        </is>
+      </c>
+      <c r="H44" t="inlineStr">
+        <is>
+          <t>low</t>
+        </is>
+      </c>
+      <c r="I44" t="inlineStr">
+        <is>
+          <t>Validation Coverage Agent</t>
+        </is>
+      </c>
+      <c r="J44" t="inlineStr">
+        <is>
+          <t>2026-06-27</t>
+        </is>
+      </c>
+      <c r="K44" t="inlineStr">
+        <is>
+          <t>Simulation Gate Authority</t>
+        </is>
+      </c>
+      <c r="L44" t="inlineStr">
+        <is>
+          <t>controlled_open</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
docs: add Stage 31A validation evidence log controls
</commit_message>
<xml_diff>
--- a/governance/risk_register.xlsx
+++ b/governance/risk_register.xlsx
@@ -2738,6 +2738,68 @@
         </is>
       </c>
     </row>
+    <row r="45">
+      <c r="A45" t="inlineStr">
+        <is>
+          <t>RISK-0044</t>
+        </is>
+      </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>Stage 31A</t>
+        </is>
+      </c>
+      <c r="C45" t="inlineStr">
+        <is>
+          <t>Validation evidence logging for Stage 30A is mistaken for command sufficiency command authenticity professional assurance or readiness evidence</t>
+        </is>
+      </c>
+      <c r="D45" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="E45" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+      <c r="F45" t="inlineStr">
+        <is>
+          <t>P2</t>
+        </is>
+      </c>
+      <c r="G45" t="inlineStr">
+        <is>
+          <t>Require command-run register rows repository-state caveat evidence-file links issue and gap links validator checks and no-overclaim wording</t>
+        </is>
+      </c>
+      <c r="H45" t="inlineStr">
+        <is>
+          <t>low</t>
+        </is>
+      </c>
+      <c r="I45" t="inlineStr">
+        <is>
+          <t>Validation Evidence Agent</t>
+        </is>
+      </c>
+      <c r="J45" t="inlineStr">
+        <is>
+          <t>2026-06-27</t>
+        </is>
+      </c>
+      <c r="K45" t="inlineStr">
+        <is>
+          <t>Simulation Gate Authority</t>
+        </is>
+      </c>
+      <c r="L45" t="inlineStr">
+        <is>
+          <t>controlled_open</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
 </worksheet>
 </file>
</xml_diff>